<commit_message>
GUA şube döküm: şubeye özel sayfalar eklendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZATs4TCBCWmFwz6XvWdCr
</commit_message>
<xml_diff>
--- a/GUA_Sube_Dokum.xlsx
+++ b/GUA_Sube_Dokum.xlsx
@@ -6,8 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Şube Özeti" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detaylı Döküm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mağusa Şube" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intech Salamis Kiosk" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Şubesiz (Bekleyen)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -16,10 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <charset val="162"/>
@@ -39,12 +44,8 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +67,11 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -82,25 +88,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,936 +507,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>GUA COFFEE COMPANY TRADING LTD (AL000151) – Şube Bazlı Özet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="45" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Şube bilgisi yalnızca fatura/irsaliye üzerinde yazan kayıtlar için doldurulmuştur; diğerleri boş bırakılmıştır. Detaylı Döküm sayfasındaki N sütunundan şube seçtikçe bu tablo otomatik güncellenir.</t>
+          <t>GUA COFFEE COMPANY TRADING LTD (AL000151) – Şube Özeti</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Şube</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fatura Adedi</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Fatura Tutarı</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>İade</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Net Tutar</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Pay %</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Şube</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Fatura Adedi</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Fatura Tutarı (Borç)</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>İade Tutarı (Alacak)</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Net Tutar</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>8925</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <f>C4-D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>E4/E$7</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mağusa Şube</t>
-        </is>
-      </c>
-      <c r="B5">
-        <f>COUNTIFS('Detaylı Döküm'!$N$7:$N$150,A5,'Detaylı Döküm'!$E$7:$E$150,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="C5" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$E$7:$E$150,'Detaylı Döküm'!$N$7:$N$150,A5)</f>
-        <v/>
-      </c>
-      <c r="D5" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$F$7:$F$150,'Detaylı Döküm'!$N$7:$N$150,A5,'Detaylı Döküm'!$C$7:$C$150,"IADE FATURANIZ")</f>
-        <v/>
+          <t>Intech Salamis Kiosk</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
         <v/>
       </c>
+      <c r="F5" s="5">
+        <f>E5/E$7</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Intech Salamis Kiosk</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>COUNTIFS('Detaylı Döküm'!$N$7:$N$150,A6,'Detaylı Döküm'!$E$7:$E$150,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="C6" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$E$7:$E$150,'Detaylı Döküm'!$N$7:$N$150,A6)</f>
-        <v/>
-      </c>
-      <c r="D6" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$F$7:$F$150,'Detaylı Döküm'!$N$7:$N$150,A6,'Detaylı Döküm'!$C$7:$C$150,"IADE FATURANIZ")</f>
-        <v/>
+          <t>Şubesi belirsiz</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>227767.11</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>13456.09</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
         <v/>
       </c>
+      <c r="F6" s="5">
+        <f>E6/E$7</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Şube belirtilmemiş (boş)</t>
-        </is>
-      </c>
-      <c r="B7">
-        <f>SUMPRODUCT(('Detaylı Döküm'!$N$7:$N$150="")*('Detaylı Döküm'!$C$7:$C$150="FATURAMIZ"))</f>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>FATURA TOPLAMI</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
+        <f>SUM(B4:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$E$7:$E$150,'Detaylı Döküm'!$C$7:$C$150,"FATURAMIZ",'Detaylı Döküm'!$N$7:$N$150,"")</f>
+      <c r="C7" s="7">
+        <f>SUM(C4:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="1">
-        <f>SUMIFS('Detaylı Döküm'!$F$7:$F$150,'Detaylı Döküm'!$C$7:$C$150,"IADE FATURANIZ",'Detaylı Döküm'!$N$7:$N$150,"")</f>
+      <c r="D7" s="7">
+        <f>SUM(D4:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="1">
-        <f>C7-D7</f>
+      <c r="E7" s="7">
+        <f>SUM(E4:E6)</f>
         <v/>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>SUM(B5:B7)</f>
+      <c r="F7" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Ödemeler (şubesiz, genel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Devreden bakiye (2026 öncesi)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>43927.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13.04.2026 – GD/282/HAVALE</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-113526.11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>28.08.2026 – GD/567/ İŞBANKASI HAVALE</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>-97623.25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Cari borç bakiyesi (dökümle aynı)</t>
+        </is>
+      </c>
+      <c r="E13" s="10">
+        <f>E7+SUM(E10:E12)</f>
         <v/>
       </c>
-      <c r="C8" s="7">
-        <f>SUM(C5:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="7">
-        <f>SUM(D5:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="7">
-        <f>SUM(E5:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Fatura Listesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Tarih</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Fiş No</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Tür</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Tutar</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Şube</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10">
-        <f>'Detaylı Döküm'!A7</f>
-        <v/>
-      </c>
-      <c r="B13">
-        <f>'Detaylı Döküm'!B7</f>
-        <v/>
-      </c>
-      <c r="C13">
-        <f>'Detaylı Döküm'!C7</f>
-        <v/>
-      </c>
-      <c r="D13" s="1">
-        <f>IF('Detaylı Döküm'!E7&gt;0,'Detaylı Döküm'!E7,-'Detaylı Döküm'!F7)</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>IF('Detaylı Döküm'!N7="","",'Detaylı Döküm'!N7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10">
-        <f>'Detaylı Döküm'!A11</f>
-        <v/>
-      </c>
-      <c r="B14">
-        <f>'Detaylı Döküm'!B11</f>
-        <v/>
-      </c>
-      <c r="C14">
-        <f>'Detaylı Döküm'!C11</f>
-        <v/>
-      </c>
-      <c r="D14" s="1">
-        <f>IF('Detaylı Döküm'!E11&gt;0,'Detaylı Döküm'!E11,-'Detaylı Döküm'!F11)</f>
-        <v/>
-      </c>
-      <c r="E14">
-        <f>IF('Detaylı Döküm'!N11="","",'Detaylı Döküm'!N11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10">
-        <f>'Detaylı Döküm'!A14</f>
-        <v/>
-      </c>
-      <c r="B15">
-        <f>'Detaylı Döküm'!B14</f>
-        <v/>
-      </c>
-      <c r="C15">
-        <f>'Detaylı Döküm'!C14</f>
-        <v/>
-      </c>
-      <c r="D15" s="1">
-        <f>IF('Detaylı Döküm'!E14&gt;0,'Detaylı Döküm'!E14,-'Detaylı Döküm'!F14)</f>
-        <v/>
-      </c>
-      <c r="E15">
-        <f>IF('Detaylı Döküm'!N14="","",'Detaylı Döküm'!N14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10">
-        <f>'Detaylı Döküm'!A17</f>
-        <v/>
-      </c>
-      <c r="B16">
-        <f>'Detaylı Döküm'!B17</f>
-        <v/>
-      </c>
-      <c r="C16">
-        <f>'Detaylı Döküm'!C17</f>
-        <v/>
-      </c>
-      <c r="D16" s="1">
-        <f>IF('Detaylı Döküm'!E17&gt;0,'Detaylı Döküm'!E17,-'Detaylı Döküm'!F17)</f>
-        <v/>
-      </c>
-      <c r="E16">
-        <f>IF('Detaylı Döküm'!N17="","",'Detaylı Döküm'!N17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10">
-        <f>'Detaylı Döküm'!A20</f>
-        <v/>
-      </c>
-      <c r="B17">
-        <f>'Detaylı Döküm'!B20</f>
-        <v/>
-      </c>
-      <c r="C17">
-        <f>'Detaylı Döküm'!C20</f>
-        <v/>
-      </c>
-      <c r="D17" s="1">
-        <f>IF('Detaylı Döküm'!E20&gt;0,'Detaylı Döküm'!E20,-'Detaylı Döküm'!F20)</f>
-        <v/>
-      </c>
-      <c r="E17">
-        <f>IF('Detaylı Döküm'!N20="","",'Detaylı Döküm'!N20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10">
-        <f>'Detaylı Döküm'!A23</f>
-        <v/>
-      </c>
-      <c r="B18">
-        <f>'Detaylı Döküm'!B23</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>'Detaylı Döküm'!C23</f>
-        <v/>
-      </c>
-      <c r="D18" s="1">
-        <f>IF('Detaylı Döküm'!E23&gt;0,'Detaylı Döküm'!E23,-'Detaylı Döküm'!F23)</f>
-        <v/>
-      </c>
-      <c r="E18">
-        <f>IF('Detaylı Döküm'!N23="","",'Detaylı Döküm'!N23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10">
-        <f>'Detaylı Döküm'!A27</f>
-        <v/>
-      </c>
-      <c r="B19">
-        <f>'Detaylı Döküm'!B27</f>
-        <v/>
-      </c>
-      <c r="C19">
-        <f>'Detaylı Döküm'!C27</f>
-        <v/>
-      </c>
-      <c r="D19" s="1">
-        <f>IF('Detaylı Döküm'!E27&gt;0,'Detaylı Döküm'!E27,-'Detaylı Döküm'!F27)</f>
-        <v/>
-      </c>
-      <c r="E19">
-        <f>IF('Detaylı Döküm'!N27="","",'Detaylı Döküm'!N27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10">
-        <f>'Detaylı Döküm'!A30</f>
-        <v/>
-      </c>
-      <c r="B20">
-        <f>'Detaylı Döküm'!B30</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>'Detaylı Döküm'!C30</f>
-        <v/>
-      </c>
-      <c r="D20" s="1">
-        <f>IF('Detaylı Döküm'!E30&gt;0,'Detaylı Döküm'!E30,-'Detaylı Döküm'!F30)</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>IF('Detaylı Döküm'!N30="","",'Detaylı Döküm'!N30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10">
-        <f>'Detaylı Döküm'!A35</f>
-        <v/>
-      </c>
-      <c r="B21">
-        <f>'Detaylı Döküm'!B35</f>
-        <v/>
-      </c>
-      <c r="C21">
-        <f>'Detaylı Döküm'!C35</f>
-        <v/>
-      </c>
-      <c r="D21" s="1">
-        <f>IF('Detaylı Döküm'!E35&gt;0,'Detaylı Döküm'!E35,-'Detaylı Döküm'!F35)</f>
-        <v/>
-      </c>
-      <c r="E21">
-        <f>IF('Detaylı Döküm'!N35="","",'Detaylı Döküm'!N35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10">
-        <f>'Detaylı Döküm'!A39</f>
-        <v/>
-      </c>
-      <c r="B22">
-        <f>'Detaylı Döküm'!B39</f>
-        <v/>
-      </c>
-      <c r="C22">
-        <f>'Detaylı Döküm'!C39</f>
-        <v/>
-      </c>
-      <c r="D22" s="1">
-        <f>IF('Detaylı Döküm'!E39&gt;0,'Detaylı Döküm'!E39,-'Detaylı Döküm'!F39)</f>
-        <v/>
-      </c>
-      <c r="E22">
-        <f>IF('Detaylı Döküm'!N39="","",'Detaylı Döküm'!N39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10">
-        <f>'Detaylı Döküm'!A42</f>
-        <v/>
-      </c>
-      <c r="B23">
-        <f>'Detaylı Döküm'!B42</f>
-        <v/>
-      </c>
-      <c r="C23">
-        <f>'Detaylı Döküm'!C42</f>
-        <v/>
-      </c>
-      <c r="D23" s="1">
-        <f>IF('Detaylı Döküm'!E42&gt;0,'Detaylı Döküm'!E42,-'Detaylı Döküm'!F42)</f>
-        <v/>
-      </c>
-      <c r="E23">
-        <f>IF('Detaylı Döküm'!N42="","",'Detaylı Döküm'!N42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10">
-        <f>'Detaylı Döküm'!A45</f>
-        <v/>
-      </c>
-      <c r="B24">
-        <f>'Detaylı Döküm'!B45</f>
-        <v/>
-      </c>
-      <c r="C24">
-        <f>'Detaylı Döküm'!C45</f>
-        <v/>
-      </c>
-      <c r="D24" s="1">
-        <f>IF('Detaylı Döküm'!E45&gt;0,'Detaylı Döküm'!E45,-'Detaylı Döküm'!F45)</f>
-        <v/>
-      </c>
-      <c r="E24">
-        <f>IF('Detaylı Döküm'!N45="","",'Detaylı Döküm'!N45)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10">
-        <f>'Detaylı Döküm'!A51</f>
-        <v/>
-      </c>
-      <c r="B25">
-        <f>'Detaylı Döküm'!B51</f>
-        <v/>
-      </c>
-      <c r="C25">
-        <f>'Detaylı Döküm'!C51</f>
-        <v/>
-      </c>
-      <c r="D25" s="1">
-        <f>IF('Detaylı Döküm'!E51&gt;0,'Detaylı Döküm'!E51,-'Detaylı Döküm'!F51)</f>
-        <v/>
-      </c>
-      <c r="E25">
-        <f>IF('Detaylı Döküm'!N51="","",'Detaylı Döküm'!N51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10">
-        <f>'Detaylı Döküm'!A57</f>
-        <v/>
-      </c>
-      <c r="B26">
-        <f>'Detaylı Döküm'!B57</f>
-        <v/>
-      </c>
-      <c r="C26">
-        <f>'Detaylı Döküm'!C57</f>
-        <v/>
-      </c>
-      <c r="D26" s="1">
-        <f>IF('Detaylı Döküm'!E57&gt;0,'Detaylı Döküm'!E57,-'Detaylı Döküm'!F57)</f>
-        <v/>
-      </c>
-      <c r="E26">
-        <f>IF('Detaylı Döküm'!N57="","",'Detaylı Döküm'!N57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10">
-        <f>'Detaylı Döküm'!A60</f>
-        <v/>
-      </c>
-      <c r="B27">
-        <f>'Detaylı Döküm'!B60</f>
-        <v/>
-      </c>
-      <c r="C27">
-        <f>'Detaylı Döküm'!C60</f>
-        <v/>
-      </c>
-      <c r="D27" s="1">
-        <f>IF('Detaylı Döküm'!E60&gt;0,'Detaylı Döküm'!E60,-'Detaylı Döküm'!F60)</f>
-        <v/>
-      </c>
-      <c r="E27">
-        <f>IF('Detaylı Döküm'!N60="","",'Detaylı Döküm'!N60)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10">
-        <f>'Detaylı Döküm'!A63</f>
-        <v/>
-      </c>
-      <c r="B28">
-        <f>'Detaylı Döküm'!B63</f>
-        <v/>
-      </c>
-      <c r="C28">
-        <f>'Detaylı Döküm'!C63</f>
-        <v/>
-      </c>
-      <c r="D28" s="1">
-        <f>IF('Detaylı Döküm'!E63&gt;0,'Detaylı Döküm'!E63,-'Detaylı Döküm'!F63)</f>
-        <v/>
-      </c>
-      <c r="E28">
-        <f>IF('Detaylı Döküm'!N63="","",'Detaylı Döküm'!N63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10">
-        <f>'Detaylı Döküm'!A70</f>
-        <v/>
-      </c>
-      <c r="B29">
-        <f>'Detaylı Döküm'!B70</f>
-        <v/>
-      </c>
-      <c r="C29">
-        <f>'Detaylı Döküm'!C70</f>
-        <v/>
-      </c>
-      <c r="D29" s="1">
-        <f>IF('Detaylı Döküm'!E70&gt;0,'Detaylı Döküm'!E70,-'Detaylı Döküm'!F70)</f>
-        <v/>
-      </c>
-      <c r="E29">
-        <f>IF('Detaylı Döküm'!N70="","",'Detaylı Döküm'!N70)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10">
-        <f>'Detaylı Döküm'!A74</f>
-        <v/>
-      </c>
-      <c r="B30">
-        <f>'Detaylı Döküm'!B74</f>
-        <v/>
-      </c>
-      <c r="C30">
-        <f>'Detaylı Döküm'!C74</f>
-        <v/>
-      </c>
-      <c r="D30" s="1">
-        <f>IF('Detaylı Döküm'!E74&gt;0,'Detaylı Döküm'!E74,-'Detaylı Döküm'!F74)</f>
-        <v/>
-      </c>
-      <c r="E30">
-        <f>IF('Detaylı Döküm'!N74="","",'Detaylı Döküm'!N74)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10">
-        <f>'Detaylı Döküm'!A77</f>
-        <v/>
-      </c>
-      <c r="B31">
-        <f>'Detaylı Döküm'!B77</f>
-        <v/>
-      </c>
-      <c r="C31">
-        <f>'Detaylı Döküm'!C77</f>
-        <v/>
-      </c>
-      <c r="D31" s="1">
-        <f>IF('Detaylı Döküm'!E77&gt;0,'Detaylı Döküm'!E77,-'Detaylı Döküm'!F77)</f>
-        <v/>
-      </c>
-      <c r="E31">
-        <f>IF('Detaylı Döküm'!N77="","",'Detaylı Döküm'!N77)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10">
-        <f>'Detaylı Döküm'!A84</f>
-        <v/>
-      </c>
-      <c r="B32">
-        <f>'Detaylı Döküm'!B84</f>
-        <v/>
-      </c>
-      <c r="C32">
-        <f>'Detaylı Döküm'!C84</f>
-        <v/>
-      </c>
-      <c r="D32" s="1">
-        <f>IF('Detaylı Döküm'!E84&gt;0,'Detaylı Döküm'!E84,-'Detaylı Döküm'!F84)</f>
-        <v/>
-      </c>
-      <c r="E32">
-        <f>IF('Detaylı Döküm'!N84="","",'Detaylı Döküm'!N84)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10">
-        <f>'Detaylı Döküm'!A87</f>
-        <v/>
-      </c>
-      <c r="B33">
-        <f>'Detaylı Döküm'!B87</f>
-        <v/>
-      </c>
-      <c r="C33">
-        <f>'Detaylı Döküm'!C87</f>
-        <v/>
-      </c>
-      <c r="D33" s="1">
-        <f>IF('Detaylı Döküm'!E87&gt;0,'Detaylı Döküm'!E87,-'Detaylı Döküm'!F87)</f>
-        <v/>
-      </c>
-      <c r="E33">
-        <f>IF('Detaylı Döküm'!N87="","",'Detaylı Döküm'!N87)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10">
-        <f>'Detaylı Döküm'!A94</f>
-        <v/>
-      </c>
-      <c r="B34">
-        <f>'Detaylı Döküm'!B94</f>
-        <v/>
-      </c>
-      <c r="C34">
-        <f>'Detaylı Döküm'!C94</f>
-        <v/>
-      </c>
-      <c r="D34" s="1">
-        <f>IF('Detaylı Döküm'!E94&gt;0,'Detaylı Döküm'!E94,-'Detaylı Döküm'!F94)</f>
-        <v/>
-      </c>
-      <c r="E34">
-        <f>IF('Detaylı Döküm'!N94="","",'Detaylı Döküm'!N94)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10">
-        <f>'Detaylı Döküm'!A97</f>
-        <v/>
-      </c>
-      <c r="B35">
-        <f>'Detaylı Döküm'!B97</f>
-        <v/>
-      </c>
-      <c r="C35">
-        <f>'Detaylı Döküm'!C97</f>
-        <v/>
-      </c>
-      <c r="D35" s="1">
-        <f>IF('Detaylı Döküm'!E97&gt;0,'Detaylı Döküm'!E97,-'Detaylı Döküm'!F97)</f>
-        <v/>
-      </c>
-      <c r="E35">
-        <f>IF('Detaylı Döküm'!N97="","",'Detaylı Döküm'!N97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10">
-        <f>'Detaylı Döküm'!A100</f>
-        <v/>
-      </c>
-      <c r="B36">
-        <f>'Detaylı Döküm'!B100</f>
-        <v/>
-      </c>
-      <c r="C36">
-        <f>'Detaylı Döküm'!C100</f>
-        <v/>
-      </c>
-      <c r="D36" s="1">
-        <f>IF('Detaylı Döküm'!E100&gt;0,'Detaylı Döküm'!E100,-'Detaylı Döküm'!F100)</f>
-        <v/>
-      </c>
-      <c r="E36">
-        <f>IF('Detaylı Döküm'!N100="","",'Detaylı Döküm'!N100)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10">
-        <f>'Detaylı Döküm'!A107</f>
-        <v/>
-      </c>
-      <c r="B37">
-        <f>'Detaylı Döküm'!B107</f>
-        <v/>
-      </c>
-      <c r="C37">
-        <f>'Detaylı Döküm'!C107</f>
-        <v/>
-      </c>
-      <c r="D37" s="1">
-        <f>IF('Detaylı Döküm'!E107&gt;0,'Detaylı Döküm'!E107,-'Detaylı Döküm'!F107)</f>
-        <v/>
-      </c>
-      <c r="E37">
-        <f>IF('Detaylı Döküm'!N107="","",'Detaylı Döküm'!N107)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10">
-        <f>'Detaylı Döküm'!A110</f>
-        <v/>
-      </c>
-      <c r="B38">
-        <f>'Detaylı Döküm'!B110</f>
-        <v/>
-      </c>
-      <c r="C38">
-        <f>'Detaylı Döküm'!C110</f>
-        <v/>
-      </c>
-      <c r="D38" s="1">
-        <f>IF('Detaylı Döküm'!E110&gt;0,'Detaylı Döküm'!E110,-'Detaylı Döküm'!F110)</f>
-        <v/>
-      </c>
-      <c r="E38">
-        <f>IF('Detaylı Döküm'!N110="","",'Detaylı Döküm'!N110)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10">
-        <f>'Detaylı Döküm'!A113</f>
-        <v/>
-      </c>
-      <c r="B39">
-        <f>'Detaylı Döküm'!B113</f>
-        <v/>
-      </c>
-      <c r="C39">
-        <f>'Detaylı Döküm'!C113</f>
-        <v/>
-      </c>
-      <c r="D39" s="1">
-        <f>IF('Detaylı Döküm'!E113&gt;0,'Detaylı Döküm'!E113,-'Detaylı Döküm'!F113)</f>
-        <v/>
-      </c>
-      <c r="E39">
-        <f>IF('Detaylı Döküm'!N113="","",'Detaylı Döküm'!N113)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10">
-        <f>'Detaylı Döküm'!A117</f>
-        <v/>
-      </c>
-      <c r="B40">
-        <f>'Detaylı Döküm'!B117</f>
-        <v/>
-      </c>
-      <c r="C40">
-        <f>'Detaylı Döküm'!C117</f>
-        <v/>
-      </c>
-      <c r="D40" s="1">
-        <f>IF('Detaylı Döküm'!E117&gt;0,'Detaylı Döküm'!E117,-'Detaylı Döküm'!F117)</f>
-        <v/>
-      </c>
-      <c r="E40">
-        <f>IF('Detaylı Döküm'!N117="","",'Detaylı Döküm'!N117)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10">
-        <f>'Detaylı Döküm'!A121</f>
-        <v/>
-      </c>
-      <c r="B41">
-        <f>'Detaylı Döküm'!B121</f>
-        <v/>
-      </c>
-      <c r="C41">
-        <f>'Detaylı Döküm'!C121</f>
-        <v/>
-      </c>
-      <c r="D41" s="1">
-        <f>IF('Detaylı Döküm'!E121&gt;0,'Detaylı Döküm'!E121,-'Detaylı Döküm'!F121)</f>
-        <v/>
-      </c>
-      <c r="E41">
-        <f>IF('Detaylı Döküm'!N121="","",'Detaylı Döküm'!N121)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10">
-        <f>'Detaylı Döküm'!A128</f>
-        <v/>
-      </c>
-      <c r="B42">
-        <f>'Detaylı Döküm'!B128</f>
-        <v/>
-      </c>
-      <c r="C42">
-        <f>'Detaylı Döküm'!C128</f>
-        <v/>
-      </c>
-      <c r="D42" s="1">
-        <f>IF('Detaylı Döküm'!E128&gt;0,'Detaylı Döküm'!E128,-'Detaylı Döküm'!F128)</f>
-        <v/>
-      </c>
-      <c r="E42">
-        <f>IF('Detaylı Döküm'!N128="","",'Detaylı Döküm'!N128)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="10">
-        <f>'Detaylı Döküm'!A131</f>
-        <v/>
-      </c>
-      <c r="B43">
-        <f>'Detaylı Döküm'!B131</f>
-        <v/>
-      </c>
-      <c r="C43">
-        <f>'Detaylı Döküm'!C131</f>
-        <v/>
-      </c>
-      <c r="D43" s="1">
-        <f>IF('Detaylı Döküm'!E131&gt;0,'Detaylı Döküm'!E131,-'Detaylı Döküm'!F131)</f>
-        <v/>
-      </c>
-      <c r="E43">
-        <f>IF('Detaylı Döküm'!N131="","",'Detaylı Döküm'!N131)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10">
-        <f>'Detaylı Döküm'!A137</f>
-        <v/>
-      </c>
-      <c r="B44">
-        <f>'Detaylı Döküm'!B137</f>
-        <v/>
-      </c>
-      <c r="C44">
-        <f>'Detaylı Döküm'!C137</f>
-        <v/>
-      </c>
-      <c r="D44" s="1">
-        <f>IF('Detaylı Döküm'!E137&gt;0,'Detaylı Döküm'!E137,-'Detaylı Döküm'!F137)</f>
-        <v/>
-      </c>
-      <c r="E44">
-        <f>IF('Detaylı Döküm'!N137="","",'Detaylı Döküm'!N137)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="10">
-        <f>'Detaylı Döküm'!A144</f>
-        <v/>
-      </c>
-      <c r="B45">
-        <f>'Detaylı Döküm'!B144</f>
-        <v/>
-      </c>
-      <c r="C45">
-        <f>'Detaylı Döküm'!C144</f>
-        <v/>
-      </c>
-      <c r="D45" s="1">
-        <f>IF('Detaylı Döküm'!E144&gt;0,'Detaylı Döküm'!E144,-'Detaylı Döküm'!F144)</f>
-        <v/>
-      </c>
-      <c r="E45">
-        <f>IF('Detaylı Döküm'!N144="","",'Detaylı Döküm'!N144)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10">
-        <f>'Detaylı Döküm'!A148</f>
-        <v/>
-      </c>
-      <c r="B46">
-        <f>'Detaylı Döküm'!B148</f>
-        <v/>
-      </c>
-      <c r="C46">
-        <f>'Detaylı Döküm'!C148</f>
-        <v/>
-      </c>
-      <c r="D46" s="1">
-        <f>IF('Detaylı Döküm'!E148&gt;0,'Detaylı Döküm'!E148,-'Detaylı Döküm'!F148)</f>
-        <v/>
-      </c>
-      <c r="E46">
-        <f>IF('Detaylı Döküm'!N148="","",'Detaylı Döküm'!N148)</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1530,7 +804,7 @@
           <t>Plasiyer Kodu</t>
         </is>
       </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>Şube</t>
         </is>
@@ -1589,7 +863,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N7" s="12" t="n"/>
+      <c r="N7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -1779,7 +1053,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N11" s="12" t="n"/>
+      <c r="N11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -1923,7 +1197,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N14" s="12" t="n"/>
+      <c r="N14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -2067,7 +1341,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N17" s="12" t="n"/>
+      <c r="N17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -2211,7 +1485,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N20" s="12" t="n"/>
+      <c r="N20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -2355,7 +1629,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N23" s="12" t="n"/>
+      <c r="N23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
@@ -2545,7 +1819,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N27" s="12" t="n"/>
+      <c r="N27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
@@ -2689,7 +1963,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N30" s="12" t="n"/>
+      <c r="N30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -2925,7 +2199,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N35" s="12" t="n"/>
+      <c r="N35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
@@ -3115,7 +2389,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N39" s="12" t="n"/>
+      <c r="N39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
@@ -3259,7 +2533,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N42" s="12" t="n"/>
+      <c r="N42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
@@ -3403,7 +2677,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N45" s="12" t="n"/>
+      <c r="N45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
@@ -3674,7 +2948,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N51" s="12" t="n"/>
+      <c r="N51" s="11" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
@@ -3956,7 +3230,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N57" s="12" t="n"/>
+      <c r="N57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
@@ -4100,7 +3374,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N60" s="12" t="n"/>
+      <c r="N60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
@@ -4244,7 +3518,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N63" s="12" t="n"/>
+      <c r="N63" s="11" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
@@ -4572,7 +3846,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N70" s="12" t="n"/>
+      <c r="N70" s="11" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
@@ -4762,7 +4036,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N74" s="12" t="n"/>
+      <c r="N74" s="11" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
@@ -4906,7 +4180,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N77" s="12" t="n"/>
+      <c r="N77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
@@ -5234,7 +4508,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N84" s="12" t="n"/>
+      <c r="N84" s="11" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
@@ -5378,7 +4652,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N87" s="12" t="n"/>
+      <c r="N87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
@@ -5706,7 +4980,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N94" s="12" t="n"/>
+      <c r="N94" s="11" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
@@ -5850,7 +5124,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N97" s="12" t="n"/>
+      <c r="N97" s="11" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
@@ -5994,7 +5268,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N100" s="12" t="n"/>
+      <c r="N100" s="11" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
@@ -6322,7 +5596,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N107" s="12" t="n"/>
+      <c r="N107" s="11" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
@@ -6466,7 +5740,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N110" s="12" t="n"/>
+      <c r="N110" s="11" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
@@ -6610,7 +5884,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N113" s="12" t="n"/>
+      <c r="N113" s="11" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
@@ -6800,7 +6074,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N117" s="12" t="n"/>
+      <c r="N117" s="11" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
@@ -6990,7 +6264,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N121" s="12" t="n"/>
+      <c r="N121" s="11" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
@@ -7307,7 +6581,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N128" s="12" t="n"/>
+      <c r="N128" s="11" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
@@ -7451,7 +6725,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N131" s="12" t="n"/>
+      <c r="N131" s="11" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
@@ -7733,7 +7007,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N137" s="12" t="n"/>
+      <c r="N137" s="11" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
@@ -8061,7 +7335,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N144" s="12" t="n"/>
+      <c r="N144" s="11" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
@@ -8251,7 +7525,7 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N148" s="13" t="inlineStr">
+      <c r="N148" s="12" t="inlineStr">
         <is>
           <t>Mağusa Şube</t>
         </is>
@@ -8404,11 +7678,1039 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="N7 N11 N14 N17 N20 N23 N27 N30 N35 N39 N42 N45 N51 N57 N60 N63 N70 N74 N77 N84 N87 N94 N97 N100 N107 N110 N113 N117 N121 N128 N131 N137 N144 N148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Mağusa Şube,Intech Salamis Kiosk"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>GUA COFFEE COMPANY TRADING LTD – Mağusa Şube</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fiş No</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Açıklama</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Vade</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Tutar (KDV dahil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>A00000000263729</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>46409</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>8925</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GUS295</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GUSTEA DEMLİK SİYAH ÇAY 12 KG</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>8925</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>TOPLAM (net)</t>
+        </is>
+      </c>
+      <c r="E7" s="10">
+        <f>E4</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>GUA COFFEE COMPANY TRADING LTD – Intech Salamis Kiosk</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fiş No</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Açıklama</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Vade</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Tutar (KDV dahil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Henüz bu şubeye eşleşen fatura yok.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Şubesi henüz belirlenmemiş faturalar (teslim fişi / şube bilgisi gerekli)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fiş No</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Tür</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Tutar</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Ürünler</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Şube (doldur)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A00000000242321</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>3960</v>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A00000000242322</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1980</v>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI FRAMBUAZ 4 KG KL/4AD x1</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A00000000242346</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>870</v>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY KONT.BAZ PLASTİK POMPASI x5</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A00000000242518</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>1190.25</v>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>PİPET KAĞIT BYZ BUBBLE 12X24 PK/75AD KL/14PK x10</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A00000000242620</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>11550</v>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>GUA İKİLİ TAŞIYICI PK/100 ADETLİ x1000</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A00000000243183</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>1291.13</v>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY KONT.BAZ PLASTİK POMPASI x4; PİPET KAĞIT BYZ BUBBLE 12X24 PK/75AD KL/14PK x5</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A00000000244577</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>33852</v>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>GUA RAMAZAN 14 OZ DW KARTON BARDAK KL/500AD x10000</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A00000000246358</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>6153.59</v>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>GUSSE MEY.PÜRE 1,1LT  YABAN MERSİNİ x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A00000000246493</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>5509.88</v>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>GUA BASKILI 22X11X28 KRAFT DÜZ SAP KL/300 x250; GUSSE MEY.PÜRE 1,1LT  BÖĞÜRTLEN x1</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A00000000246753</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>4158</v>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>GUSSE MEY.PÜRE 1,1LT  BÖĞÜRTLEN x6</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>I00000000246861</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>IADE FATURANIZ</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>-916.49</v>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>GUSSE MEY.PÜRE 1,1LT  YABAN MERSİNİ x1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>A00000000248046</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>8118</v>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>GUSSE MEY.PÜRE 1,1LT  BÖĞÜRTLEN x6; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>A00000000249366</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>7920</v>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY TOPLARI MANGO 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>A00000000250156</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>3960</v>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x2</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>A00000000250895</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>5780.25</v>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>GUA BASKILI 22X11X28 KRAFT DÜZ SAP KL/300 x300</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>A00000000251139</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>8910</v>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI MANGO 4KG KL/4AD (2.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x1; BOBAJOY MEYVE SUYU TOPLARI FRAMBUAZ 4 KG KL/4AD x1</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>A00000000251140</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>1980</v>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>A00000000252956</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>1980</v>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A00000000253718</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>9900</v>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY TOPLARI MANGO 4KG KL/4AD (2.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>A00000000254148</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>1980</v>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A00000000254821</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>19469.6</v>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI MANGO 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x1; BİO PİPET BEYAZ 7X22  PK/250AD KL/20 PK x40</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A00000000254951</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>12992</v>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20 x40</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>I00000000255472</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>IADE FATURANIZ</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>-12539.6</v>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>BİO PİPET BEYAZ 7X22  PK/250AD KL/20 PK x40</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>A00000000255781</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>14250</v>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>GUA BASKILI 22X11X28 KRAFT DÜZ SAP KL/300 x600; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x3; TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A00000000255791</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>495</v>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI Y.MERSİNİ 1KG KL/12AD x1</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>A00000000256524</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>4640</v>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>PİPET KAĞIT BEYAZ 12X21 SARGILI PK/200AD KL/10PK x10</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>A00000000257286</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>1848</v>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x1</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>A00000000257723</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>5940</v>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x2; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>A00000000259067</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>7920</v>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>A00000000259115</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>1848</v>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F33" s="18" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>A00000000259123</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>20481.41</v>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x2; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20 x40; TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x2</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>A00000000259190</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>13285</v>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 6X23 SARGILI PK/200AD KL/25 x25</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>A00000000263425</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>3555</v>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; 14 OZ BEYAZ DÜZ KAPAK KL/1000 x1000</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="n"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>TOPLAM (net)</t>
+        </is>
+      </c>
+      <c r="D38" s="1">
+        <f>SUM(D4:D36)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
GUA şube döküm: 259123 Mağusa'ya eşlendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZATs4TCBCWmFwz6XvWdCr
</commit_message>
<xml_diff>
--- a/GUA_Sube_Dokum.xlsx
+++ b/GUA_Sube_Dokum.xlsx
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>8925</v>
+        <v>29406.41</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>227767.11</v>
+        <v>207285.7</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>13456.09</v>
@@ -6725,7 +6725,11 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N131" s="11" t="inlineStr"/>
+      <c r="N131" s="12" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
@@ -7688,7 +7692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7734,11 +7738,11 @@
     </row>
     <row r="4">
       <c r="A4" s="13" t="n">
-        <v>46319</v>
+        <v>46263</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>A00000000263729</t>
+          <t>A00000000259123</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -7747,40 +7751,141 @@
         </is>
       </c>
       <c r="D4" s="13" t="n">
-        <v>46409</v>
+        <v>46353</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>8925</v>
+        <v>20481.41</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
+          <t>ATM038</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2-AD</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>3960</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ATM040</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PTS038</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>40-PK</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>12561.41</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ATM074</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2-AD</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>A00000000263729</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>46409</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>8925</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
           <t>GUS295</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>GUSTEA DEMLİK SİYAH ÇAY 12 KG</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>1-AD</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E10" s="1" t="n">
         <v>8925</v>
       </c>
     </row>
-    <row r="7">
-      <c r="C7" s="9" t="inlineStr">
+    <row r="12">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>TOPLAM (net)</t>
         </is>
       </c>
-      <c r="E7" s="10">
-        <f>E4</f>
+      <c r="E12" s="10">
+        <f>E4+E9</f>
         <v/>
       </c>
     </row>
@@ -7857,7 +7962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8629,11 +8734,11 @@
     </row>
     <row r="34">
       <c r="A34" s="16" t="n">
-        <v>46263</v>
+        <v>46266</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>A00000000259123</t>
+          <t>A00000000259190</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -8642,22 +8747,22 @@
         </is>
       </c>
       <c r="D34" s="1" t="n">
-        <v>20481.41</v>
+        <v>13285</v>
       </c>
       <c r="E34" s="17" t="inlineStr">
         <is>
-          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x2; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20 x40; TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x2</t>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 6X23 SARGILI PK/200AD KL/25 x25</t>
         </is>
       </c>
       <c r="F34" s="18" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="n">
-        <v>46266</v>
+        <v>46315</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>A00000000259190</t>
+          <t>A00000000263425</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -8666,47 +8771,23 @@
         </is>
       </c>
       <c r="D35" s="1" t="n">
-        <v>13285</v>
+        <v>3555</v>
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 6X23 SARGILI PK/200AD KL/25 x25</t>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; 14 OZ BEYAZ DÜZ KAPAK KL/1000 x1000</t>
         </is>
       </c>
       <c r="F35" s="18" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>A00000000263425</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>3555</v>
-      </c>
-      <c r="E36" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; 14 OZ BEYAZ DÜZ KAPAK KL/1000 x1000</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="n"/>
-    </row>
-    <row r="38">
-      <c r="C38" s="9" t="inlineStr">
+    <row r="37">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>TOPLAM (net)</t>
         </is>
       </c>
-      <c r="D38" s="1">
-        <f>SUM(D4:D36)</f>
+      <c r="D37" s="1">
+        <f>SUM(D4:D35)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
GUA şube döküm: zip'teki teslim fişlerinden 10 fatura şubeye eşlendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZATs4TCBCWmFwz6XvWdCr
</commit_message>
<xml_diff>
--- a/GUA_Sube_Dokum.xlsx
+++ b/GUA_Sube_Dokum.xlsx
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>29406.41</v>
+        <v>52346.41</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0</v>
+        <v>24901</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>0</v>
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>207285.7</v>
+        <v>159444.7</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>13456.09</v>
@@ -712,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N152"/>
+  <dimension ref="A1:O152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -725,6 +725,7 @@
     <col width="9.6640625" bestFit="1" customWidth="1" min="12" max="12"/>
     <col width="11.6640625" bestFit="1" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -809,6 +810,11 @@
           <t>Şube</t>
         </is>
       </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Not (kaynak)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
@@ -864,6 +870,7 @@
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -1054,6 +1061,7 @@
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -1198,6 +1206,7 @@
         </is>
       </c>
       <c r="N14" s="11" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -1342,6 +1351,7 @@
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -1486,6 +1496,7 @@
         </is>
       </c>
       <c r="N20" s="11" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -1630,6 +1641,7 @@
         </is>
       </c>
       <c r="N23" s="11" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
@@ -1820,6 +1832,7 @@
         </is>
       </c>
       <c r="N27" s="11" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
@@ -1964,6 +1977,7 @@
         </is>
       </c>
       <c r="N30" s="11" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -2200,6 +2214,7 @@
         </is>
       </c>
       <c r="N35" s="11" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
@@ -2390,6 +2405,7 @@
         </is>
       </c>
       <c r="N39" s="11" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
@@ -2534,6 +2550,7 @@
         </is>
       </c>
       <c r="N42" s="11" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
@@ -2678,6 +2695,7 @@
         </is>
       </c>
       <c r="N45" s="11" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
@@ -2949,6 +2967,7 @@
         </is>
       </c>
       <c r="N51" s="11" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
@@ -3231,6 +3250,7 @@
         </is>
       </c>
       <c r="N57" s="11" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
@@ -3375,6 +3395,7 @@
         </is>
       </c>
       <c r="N60" s="11" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
@@ -3519,6 +3540,7 @@
         </is>
       </c>
       <c r="N63" s="11" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
@@ -3847,6 +3869,7 @@
         </is>
       </c>
       <c r="N70" s="11" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
@@ -4037,6 +4060,7 @@
         </is>
       </c>
       <c r="N74" s="11" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
@@ -4181,6 +4205,7 @@
         </is>
       </c>
       <c r="N77" s="11" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
@@ -4509,6 +4534,7 @@
         </is>
       </c>
       <c r="N84" s="11" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
@@ -4653,6 +4679,7 @@
         </is>
       </c>
       <c r="N87" s="11" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
@@ -4981,6 +5008,7 @@
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
@@ -5125,6 +5153,7 @@
         </is>
       </c>
       <c r="N97" s="11" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
@@ -5268,7 +5297,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N100" s="11" t="inlineStr"/>
+      <c r="N100" s="12" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Teslim fişi: Mağusa Şube (elle yazılı; fişte fatura no boş, kalemler eşleşiyor)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
@@ -5596,7 +5634,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N107" s="11" t="inlineStr"/>
+      <c r="N107" s="12" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>255781 ile aynı fişte (ATM057 kalemi) – Mağusa Şube; fişte fatura no yok</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
@@ -5740,7 +5787,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N110" s="11" t="inlineStr"/>
+      <c r="N110" s="12" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA ŞUBE</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
@@ -5884,7 +5940,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N113" s="11" t="inlineStr"/>
+      <c r="N113" s="12" t="inlineStr">
+        <is>
+          <t>Intech Salamis Kiosk</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Teslim fişi: KİOSK</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
@@ -6075,6 +6140,11 @@
         </is>
       </c>
       <c r="N117" s="11" t="inlineStr"/>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Fiş var ama 'Teslim Şubesi' boş bırakılmış</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
@@ -6264,7 +6334,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N121" s="11" t="inlineStr"/>
+      <c r="N121" s="12" t="inlineStr">
+        <is>
+          <t>Intech Salamis Kiosk</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
@@ -6581,7 +6660,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N128" s="11" t="inlineStr"/>
+      <c r="N128" s="12" t="inlineStr">
+        <is>
+          <t>Intech Salamis Kiosk</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
@@ -6730,6 +6818,11 @@
           <t>Mağusa Şube</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MERKEZ MAĞUSA ŞUBESİ</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
@@ -7011,7 +7104,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N137" s="11" t="inlineStr"/>
+      <c r="N137" s="12" t="inlineStr">
+        <is>
+          <t>Intech Salamis Kiosk</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
@@ -7339,7 +7441,16 @@
           <t>MRK</t>
         </is>
       </c>
-      <c r="N144" s="11" t="inlineStr"/>
+      <c r="N144" s="12" t="inlineStr">
+        <is>
+          <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA ŞUBESİ</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
@@ -7532,6 +7643,11 @@
       <c r="N148" s="12" t="inlineStr">
         <is>
           <t>Mağusa Şube</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA</t>
         </is>
       </c>
     </row>
@@ -7692,7 +7808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7700,6 +7816,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7735,14 +7852,19 @@
           <t>Tutar (KDV dahil)</t>
         </is>
       </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Not (kaynak)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="n">
-        <v>46263</v>
+        <v>46223</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>A00000000259123</t>
+          <t>A00000000255781</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -7751,41 +7873,46 @@
         </is>
       </c>
       <c r="D4" s="13" t="n">
-        <v>46353</v>
+        <v>46313</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>20481.41</v>
+        <v>14250</v>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: Mağusa Şube (elle yazılı; fişte fatura no boş, kalemler eşleşiyor)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>ATM038</t>
+          <t>MRS0010</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.)</t>
+          <t>GUA BASKILI 22X11X28 KRAFT DÜZ SAP KL/300</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2-AD</t>
+          <t>600-AD</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>3960</v>
+        <v>5670</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATM040</t>
+          <t>ATM017</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD</t>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -7800,92 +7927,381 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>PTS038</t>
+          <t>ATM033</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20</t>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>40-PK</t>
+          <t>1-AD</t>
         </is>
       </c>
       <c r="E7" s="1" t="n">
-        <v>12561.41</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
+          <t>ATM070</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3-AD</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>2772</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
           <t>ATM074</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>2-AD</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E9" s="1" t="n">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>A00000000255791</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>495</v>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>255781 ile aynı fişte (ATM057 kalemi) – Mağusa Şube; fişte fatura no yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ATM057</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI Y.MERSİNİ 1KG KL/12AD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>A00000000256524</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>4640</v>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA ŞUBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CK001</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PİPET KAĞIT BEYAZ 12X21 SARGILI PK/200AD KL/10PK</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>10-PK</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>4640</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>A00000000259123</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>46353</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>20481.41</v>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MERKEZ MAĞUSA ŞUBESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ATM038</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2-AD</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>3960</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ATM040</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="n">
         <v>1980</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="13" t="n">
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PTS038</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BİO PİPET BEYAZ 8X24 SARGILI PK/250AD KL/20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>40-PK</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>12561.41</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ATM074</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2-AD</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>A00000000263425</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>46405</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>3555</v>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA ŞUBESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ATM033</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BBT028</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14 OZ BEYAZ DÜZ KAPAK KL/1000</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>1000-AD</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n">
         <v>46319</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>A00000000263729</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>FATURAMIZ</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D22" s="13" t="n">
         <v>46409</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E22" s="15" t="n">
         <v>8925</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: MAĞUSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
         <is>
           <t>GUS295</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>GUSTEA DEMLİK SİYAH ÇAY 12 KG</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>1-AD</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E23" s="1" t="n">
         <v>8925</v>
       </c>
     </row>
-    <row r="12">
-      <c r="C12" s="9" t="inlineStr">
+    <row r="25">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>TOPLAM (net)</t>
         </is>
       </c>
-      <c r="E12" s="10">
-        <f>E4+E9</f>
+      <c r="E25" s="10">
+        <f>E4+E10+E12+E14+E19+E22</f>
         <v/>
       </c>
     </row>
@@ -7900,7 +8316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7908,6 +8324,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7943,12 +8360,365 @@
           <t>Tutar (KDV dahil)</t>
         </is>
       </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Not (kaynak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>A00000000257286</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>1848</v>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: KİOSK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Henüz bu şubeye eşleşen fatura yok.</t>
-        </is>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ATM074</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ATM070</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>A00000000259067</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>46352</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>7920</v>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ATM017</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ATM040</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ATM038</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ATM030</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>A00000000259115</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>46353</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>1848</v>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ATM070</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2-AD</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>A00000000259190</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>FATURAMIZ</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>46356</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>13285</v>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Teslim fişi: INTECH SALAMIS KIOSK ŞUBESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ATM017</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ATM038</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ATM030</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ATM040</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1-AD</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PTS032</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BİO PİPET BEYAZ 6X23 SARGILI PK/200AD KL/25</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>25-PK</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>5365</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>TOPLAM (net)</t>
+        </is>
+      </c>
+      <c r="E21" s="10">
+        <f>E4+E7+E12+E14</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -7962,7 +8732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7971,6 +8741,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8011,6 +8782,11 @@
           <t>Şube (doldur)</t>
         </is>
       </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="n">
@@ -8035,6 +8811,7 @@
         </is>
       </c>
       <c r="F4" s="18" t="n"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="n">
@@ -8059,6 +8836,7 @@
         </is>
       </c>
       <c r="F5" s="18" t="n"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="n">
@@ -8083,6 +8861,7 @@
         </is>
       </c>
       <c r="F6" s="18" t="n"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
@@ -8107,6 +8886,7 @@
         </is>
       </c>
       <c r="F7" s="18" t="n"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="n">
@@ -8131,6 +8911,7 @@
         </is>
       </c>
       <c r="F8" s="18" t="n"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
@@ -8155,6 +8936,7 @@
         </is>
       </c>
       <c r="F9" s="18" t="n"/>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="n">
@@ -8179,6 +8961,7 @@
         </is>
       </c>
       <c r="F10" s="18" t="n"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
@@ -8203,6 +8986,7 @@
         </is>
       </c>
       <c r="F11" s="18" t="n"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n">
@@ -8227,6 +9011,7 @@
         </is>
       </c>
       <c r="F12" s="18" t="n"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
@@ -8251,6 +9036,7 @@
         </is>
       </c>
       <c r="F13" s="18" t="n"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="n">
@@ -8275,6 +9061,7 @@
         </is>
       </c>
       <c r="F14" s="18" t="n"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
@@ -8299,6 +9086,7 @@
         </is>
       </c>
       <c r="F15" s="18" t="n"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n">
@@ -8323,6 +9111,7 @@
         </is>
       </c>
       <c r="F16" s="18" t="n"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n">
@@ -8347,6 +9136,7 @@
         </is>
       </c>
       <c r="F17" s="18" t="n"/>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="n">
@@ -8371,6 +9161,7 @@
         </is>
       </c>
       <c r="F18" s="18" t="n"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n">
@@ -8395,6 +9186,7 @@
         </is>
       </c>
       <c r="F19" s="18" t="n"/>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="n">
@@ -8419,6 +9211,7 @@
         </is>
       </c>
       <c r="F20" s="18" t="n"/>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="n">
@@ -8443,6 +9236,7 @@
         </is>
       </c>
       <c r="F21" s="18" t="n"/>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="n">
@@ -8467,6 +9261,7 @@
         </is>
       </c>
       <c r="F22" s="18" t="n"/>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n">
@@ -8491,6 +9286,7 @@
         </is>
       </c>
       <c r="F23" s="18" t="n"/>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="n">
@@ -8515,6 +9311,7 @@
         </is>
       </c>
       <c r="F24" s="18" t="n"/>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="n">
@@ -8539,6 +9336,7 @@
         </is>
       </c>
       <c r="F25" s="18" t="n"/>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="n">
@@ -8563,14 +9361,15 @@
         </is>
       </c>
       <c r="F26" s="18" t="n"/>
+      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n">
-        <v>46223</v>
+        <v>46245</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>A00000000255781</t>
+          <t>A00000000257723</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -8579,215 +9378,28 @@
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>14250</v>
+        <v>5940</v>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>GUA BASKILI 22X11X28 KRAFT DÜZ SAP KL/300 x600; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x3; TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x2</t>
+          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x2; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1</t>
         </is>
       </c>
       <c r="F27" s="18" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="n">
-        <v>46223</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>A00000000255791</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>495</v>
-      </c>
-      <c r="E28" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY MEYVE SUYU TOPLARI Y.MERSİNİ 1KG KL/12AD x1</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="n"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Fiş var ama 'Teslim Şubesi' boş bırakılmış</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="n">
-        <v>46230</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>A00000000256524</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>4640</v>
-      </c>
-      <c r="E29" s="17" t="inlineStr">
-        <is>
-          <t>PİPET KAĞIT BEYAZ 12X21 SARGILI PK/200AD KL/10PK x10</t>
-        </is>
-      </c>
-      <c r="F29" s="18" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="16" t="n">
-        <v>46240</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>A00000000257286</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>1848</v>
-      </c>
-      <c r="E30" s="17" t="inlineStr">
-        <is>
-          <t>TEAJOY MR.ORGO (MANGO&amp;PRTKL) 2,5 KG KL/4AD x1; TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x1</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="n">
-        <v>46245</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>A00000000257723</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>5940</v>
-      </c>
-      <c r="E31" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x2; BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="16" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>A00000000259067</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>7920</v>
-      </c>
-      <c r="E32" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1</t>
-        </is>
-      </c>
-      <c r="F32" s="18" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="16" t="n">
-        <v>46263</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>A00000000259115</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>1848</v>
-      </c>
-      <c r="E33" s="17" t="inlineStr">
-        <is>
-          <t>TEAJOY HYPE &amp; JOY (HİBİSKUS) 2,5 KG KL/4AD x2</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="n">
-        <v>46266</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>A00000000259190</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>13285</v>
-      </c>
-      <c r="E34" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY MEYVE TOPLARI ÇİLEK 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU Y.MERSİNİ 4KG KL/4AD (3.) x1; BOBAJOY MEYVE SUYU TOPLARI YEŞİL ELMA 4KG KL/4AD (2.) x1; BOBAJOY MEYVE SUYU TOPLARI MANGO 4KG KL/4AD x1; BİO PİPET BEYAZ 6X23 SARGILI PK/200AD KL/25 x25</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="16" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>A00000000263425</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>FATURAMIZ</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>3555</v>
-      </c>
-      <c r="E35" s="17" t="inlineStr">
-        <is>
-          <t>BOBAJOY TOPLARI KARAMEL 4 KG KL/4AD (3.) x1; 14 OZ BEYAZ DÜZ KAPAK KL/1000 x1000</t>
-        </is>
-      </c>
-      <c r="F35" s="18" t="n"/>
-    </row>
-    <row r="37">
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>TOPLAM (net)</t>
         </is>
       </c>
-      <c r="D37" s="1">
-        <f>SUM(D4:D35)</f>
+      <c r="D29" s="1">
+        <f>SUM(D4:D27)</f>
         <v/>
       </c>
     </row>

</xml_diff>